<commit_message>
docs: save final backfilled gpt-oss-20b responses with 5000+ chars per question
</commit_message>
<xml_diff>
--- a/data/benchmark/SEBI_Compliance_AI_Benchmark_Deliverable_A_Full_latest.xlsx
+++ b/data/benchmark/SEBI_Compliance_AI_Benchmark_Deliverable_A_Full_latest.xlsx
@@ -3702,30 +3702,33 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>**SEBI (PIT) Regulations – Disclosure &amp; Timing for an Insider Transaction**
-| Step | Who is responsible | What must be filed / disclosed | Required timeline (from the trade date) |
-|------|-------------------|--------------------------------|------------------------------------------|
-| **1. Execution of trade** | CFO (insider) | - Buy 15 Lacs worth of equity shares in the open market. | – Immediate (no delay) |
-| **2. Insider’s trade‑report** | CFO | • **Form 1** – “Insider’s transaction in the open market” (see SEBI(2020) Rules, Sect. 6) &lt;br&gt;• Must state date, time, price, quantity and nature of the transaction. | **Within 15 calendar days** of the trade |
-| **3. Transfer of report to company** | CFO | • Copy of Form 1 (or equivalent transaction report) to the company’s Board/SEC committee. | **Within 15 calendar days** of the trade |
-| **4. Company‑level disclosure** | Company (often through the IR/CSO) | • Public statement/press release on its website &amp; corporate filing portal. &lt;br&gt;• Submission of the transaction report to the securities exchange (and SEBI, if required). &lt;br&gt;• The company’s directors register must be updated (separate Companies Act requirement). | **Within 15 calendar days** of the trade (same window as insider’s reporting) |
-| **5. SEBI/Exchange filing** | Company | • The consolidated transaction report (usually the CFO’s Form 1) must be filed with the relevant exchange/SEBI under the “Insider‑Transaction” schedule of Rule‑4A of SEBI(2019) Regulations. | **Within 15 calendar days** of the trade |
-### Why these timelines apply
-* **SEBI (PIT) Reg. § 6** – “Insiders” (including CFOs, directors, promoters etc.) who buy or sell shares in the open market **must report** the transaction to the company and *within 15 days* to the exchange/SEBI.  
-* **Companies Act, 2013 – Art. 18(2)** – Disclosing any transaction by a “disclosing insider” must be made public within 15 days (and must appear in the directors’ register).  
-* **Threshold** – Because the transaction exceeds **₹15 Lac (&gt;₹1 Lac threshold)** and is in the open market, it is *mandatory* to file.  
-### Practical sequence for the CFO
-1. **On Monday** – Complete the purchase.  
-2. **Immediately / by start of next trading week** – Prepare Form 1 with all details.  
-3. **By the 15th calendar day after the trade** – Send Form 1 to the company.  
-4. **Company’s responsibility (within the same 15‑day window)**  
-   * Post the transaction in a public statement/press release.  
-   * File the report with the NSE/BSE (or the applicable exchange).  
-   * Ensure SEBI receives the filing (typically via the exchange portal).  
-If the CFO’s trade were to be made **after** the open‑market window or were a *block trade*, the same 15‑day rule applies; only the “open‑market” phrasing here changes nothing about the compliance.
----
-**Bottom line:**  
-*The CFO must file the trade report (Form 1) with the company and SEBI within 15 days of the Monday purchase, and the company must make a public disclosure and file the same with the exchange (and thereby SEBI) within the 15‑day window.*</t>
+          <t>**SEBI – Private Investment in Public Company (PIT) Regulations**
+The CFO’s purchase of her own‑company shares is a *private investment* and, because the buyer is an insider, it must be reported under the SEBI (PIT) Regulations as well as the related “Listing Obligations and Disclosure Requirements” (LODR) regime.  
+Below are the exact steps that the CFO and the company need to take, together with the time‑frames set out in the regulations.
+| Step | What must be done | Form / Notice | Required by | Time‑frame |
+|------|------------------|---------------|-------------|------------|
+| **1. Record the transaction** | The CFO must keep a written record of the buy‑back (date, price, quantity, total consideration). | – | – | – |
+| **2. File Form‑24 in the Company’s Shareholding Register** | An *Insider‑Transaction Disclosure* (Form‑24) that details: &lt;br&gt;• Total number of shares bought, &lt;br&gt;• Purchase price, &lt;br&gt;• Date of purchase, &lt;br&gt;• Total consideration, &lt;br&gt;• Whether the shares are bought on D‑/E‑P (Discount/Ex‑Price) or in the regular market. | **Form‑24** | SEBI (PIT) Regulations – “Disclosures by a private investor” | **Within 10 days of the transaction** |
+| **3. Public announcement on the Stock‑Exchange portal** | The transaction must be announced in the “Insider‑Transactions” section of the Exchange (e.g., NSE/BSE). | – | SEBI (LODR) – “Disclosure of Insider Transactions” | **Within the next trading day** after the transaction |
+| **4. Inclusion in the Company’s Periodic Information Disclosure (PID)** | The transaction must be included as a *Large Insider Transaction* in the company’s quarterly report (QIR) or the next annual report (AR). | – | SEBI (LODR) – “Large Transactions of Insiders” | **Within the next quarterly reporting cycle** (i.e., in the next QIR) |
+| **5. Update the Company’s *Annual Return* / *Form‑C*** | The transaction must be reflected in the annual return filed with the Registrar of Companies (ROC) and in the *Form‑C* (for companies) or *Form‑15E* (for government companies). | – | Companies Act &amp; SEBI | **Within the filing deadline of the annual return (within 30 days of year‑end)** |
+| **6. If the purchase crosses a material threshold** | If, in the prior 7 consecutive trading days, the cumulative acquisition is ≥ 10 % of the company’s equity or the value of the transaction is ≥ Rs 10 lakhs (whichever is lower) – *or* if the purchase raises the insider’s holding above 10 % – the company must lodge a *Notice of Transfer* and a *Large‑Transaction Notice* with the exchange and SEBI. | **Notice of Transfer (Form‑19)** and **Large‑Transaction Notice** | SEBI (PIT) &amp; LODR | **Within 24 hours** of concluding the transaction |
+| **7. Insider‑Trading compliance** | The CFO must ensure the transaction is compliant with the *Insider‑Trading* rules (no trade in restricted periods, no misuse of PPI). | – | SEBI (Prohibition of Insider Trading) Regulations | Throughout |
+| **8. Documentation &amp; audit trail** | The company must preserve all documents (trade confirmation, broker statements, filing receipts) for a minimum of 10 years as per SEBI audit requirements. | – | SEBI, Companies Act | Ongoing |
+### Quick‑Reference Timeline
+| Event | Deadline (relative to transaction day) |
+|-------|----------------------------------------|
+| **Form‑24 filed** | Within **10 days** |
+| **Exchange announcement** | Within **the next trading day** |
+| **Quarterly report inclusion** | In the **next quarterly report** |
+| **Annual return / Form‑C inclusion** | Before **year‑end annual return deadline (30 days after year‑end)** |
+| **Large‑transaction (if applicable)** | Within **24 hours** of the transaction |
+---
+### Why These Steps Matter
+1. **Transparency** – Public disclosure protects other shareholders from information asymmetry.  
+2. **Regulatory compliance** – Failure to file within the stipulated time‑frames can result in penalties (up to ₹10 lakhs and/or imprisonment for up to 3 years under SEBI).  
+3. **Insider‑trading safeguards** – The disclosure regime also serves as a deterrent to potential misuse of PPI.
+By following the table above, the CFO and the company will satisfy all SEBI (PIT) and LODR requirements associated with a private insider purchase of ₹15 lakhs in equity shares.</t>
         </is>
       </c>
       <c r="K22" t="n">
@@ -3879,14 +3882,13 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>**Immediate regulatory consequences for Acquirer A under SEBI SAST Regulations, 2011**
-| What happened | Threshold crossed | SAST‑specific duty | Deadline | Notes / Further implications |
-|---------------|------------------|-------------------|----------|------------------------------|
-| **Acquirer A already owned 22 % of voting shares in T** | &gt; 20 % (and &lt; 25 %) | A **SAST‑1** filing was required at that time (the original 22 % acquisition). | Within 5 calendar days of the original acquisition (already complied). | If not already filed, a penalty under Section 4(2) of the SAST Regulations would be imposed. |
-| **On 10 April, Acquirer A purchases an additional 4 % via block deal** | Holding rises to 26 % (22 % + 4 %) – **&gt; 25 %** | 1. **SAST‑1** (for the 4 % block deal) must be filed within 5 days (by **15 April**). &lt;br&gt;2. Because the cumulative holding now exceeds 25 %, a **mandatory takeover offer** is triggered under the SEBI (Takeovers) Regulations. Consequently, Acquirer A must file a **SAST‑2** (or equivalent notification) to disclose the intention to make a takeover offer and to comply with the takeover‐code provisions. | 1. 5 days from the block‑deal (15 April). &lt;br&gt;2. For the takeover offer – a 21‑day window to make the offer after acquiring 25 % (i.e., by 30 April) if the intent is to acquire 51 % or more. | **Exchange &amp; SEBI disclosure** – The SAST‑1 is submitted to the stock exchange (NSE/BSE) which immediately publishes the details and forwards the data to SEBI. The 4 % block‑deal must also be reported as a block‑deal to the exchange, and the target company’s board will be notified. |
-| **Other compliance** |  | • Any subsequent purchase or sale that changes the cumulative holding must be reported through the same channels. &lt;br&gt;• If Acquirer A intends to keep the holding at 26 % (i.e., not to acquire 51 %), it is **still subject to takeover‑code disclosure** and must keep the shareholders informed. | | |
-### Key Take‑away
-1. **SAST‑1 filing is mandatory within 5 days** of the block‑deal; the filing must contain</t>
+          <t>**Immediate SEBI SAST‑Regulation compliance on 10 April**
+| Step | What it is | What the law says | Where it is reported | Timeline |
+|------|------------|-------------------|----------------------|----------|
+| **1. Block‑deal reporting** | The 4 % purchase (block deal) is a transaction that exceeds **5 %** of the target’s total issued shares. | SEBI (Share Acquisition and Disclosure) Regulations, 2011 – Reg. 3 (Block‑deal reporting). | 1) To the exchange (NSE/BSE) as part of the *Block‑Deal Report*; 2) To the company via a Notice of Acquisition (Form F‑5 in the Exchange‑Listing‐Obligations scheme). | Within 30 days of the transaction; most exchanges also require the report within the same trading day or, at the latest, 3 days after the trade. |
+| **2. Share‑Acquisition Report (SAR)** | Acquirer A’s aggregate voting‑rights holding in T has risen from **22 %** to **26 %** – crossing the **15 %** threshold. | Reg. 6 (mandatory reporting of shareholding). 5 % or more = SAR (Form F‑6); 15 % or more = “Large‑shareholder” status. | To SEBI by uploading the SAR on the SEBI portal/Exchange data feed. | Within 30 days of acquisition (by 9 May 2026). |
+| **3. Disclosure of updated holding** | The new 26 % stake must be disclosed publicly as part of the shareholding pattern. | SEBI‑Reg. 5 (quarterly reporting) and Companies Act, 2013 – Section 127/128. | 1) Company publishes updated shareholding on its website/ in the next quarterly report (Form 3F). 2) Investor displays the holding in his register. | By the next reporting deadline (typically within the same quarter). |
+| **4. (Future implication) Tender‑offer trigger** | Holding ≥15 % of voting shares creates an obligation to make a tender offer if the investor wishes to acquire more than 15 %. |  SEBI (Tender Offer) Regulations</t>
         </is>
       </c>
       <c r="K23" t="n">
@@ -5388,14 +5390,25 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Below is a “walk‑through” that shows every regulatory touch‑point the company (P) must honour while:
-* **Issuing a rights‑issue of ₹500 Cr** (a primary equity raising),
-* **Facing a hostile open‑offer (SAST‑takeover)** from an external acquirer (A), and
-* **Having just received CDSCO (Drug Controller General of India) approval** for a blockbuster drug (UPSI).
-Because the three events unfold in near‑contemporaneous window, some filings overlap and some triggers a follow‑up action after the first event is complete.  The chart below breaks down what must be done under each of the four key regulatory regimes:
-| Regime | Trigger | Key Obligation(s) | Who must file/notify? | Time‑frame |
-|--------|---------|-------------------|-----------------------|------------|
-| **ICDR** (Insolvency &amp; Corporate Debt Restructuring) | • Any debt‑equity swap or capital raising that could materially impact creditors.&lt;br&gt;• New equity issuances when the company has existing defaulting debt or is in distress.&lt;br&gt;• *If* the rights‑issue is treated as a “debt‑restructuring” (e.g. paying off other creditors). | 1. **Committee of Creditors (CoC) approval** if the issuance is a “debt‑to‑equity swap” or the company has 50 %+ default default holdings.&lt;br&gt;2. **File a notice** with the ICDR tribunal if the capital raising could be considered a “restructuring” that would change the creditors’ position.&lt;br&gt;3.</t>
+          <t>### 1.  Context &amp; The 4 Regulatory Pillars
+| Framework | Key Purpose | Typical Documents / Forms |
+|-----------|-------------|---------------------------|
+| **ICDR** *(In‑centive Corporate Disclosure Rules &amp; Corporate Governance)* | Ensures that every material corporate event is disclosed transparently and in a timely manner.  Governs board approval, conflict‑of‑interest, independent audit and disclosure guidelines. | **Board Resolutions**, **Audit Committee Minutes**, **Special Form FRM‑L01**, **Special Form FRD‑1**, **ICDR‑Disclosure Schedule** |
+| **SAST** *(Securities and Take‑over Act / Transfer Regulations – commonly referred to as “SAST” in India)* | Regulates **hostile open offers** (take‑over bids).  Sets the threshold for when an offer must be made, price‑fairness, and disclosure of bid valuation, holdings etc. | **Offer Letter**, **Fairness Rating Report (FRR)**, **Form 27/28** (for SEBI filing), **Public Disclosure of Offer Schedule** |
+| **LODR** *(Listing Obligations &amp; Disclosure Requirements – SEBI)* | Lists all the specific disclosures a SEBI‑listed entity must make when it plans a rights issue, a change in share capital, or any material event. | **Form FRM‑L01** (rights issue notice), **Form FRM‑C01** (offer letter), **Form FRD‑1** (material event), **Continuous Disclosure Notice (CDN)** |
+| **PIT** *(Price‑Impact Test – part of LODR &amp; SEBI rules)* | Requires a detailed, independent price‑impact analysis before any public issue or rights issue to confirm the proposal price isn’t detrimental to the market. | **PIT Report** (valuation, benchmarking, audit), attached to **Form FRM‑L01** |
+Below is a step‑by‑step walkthrough of the compliance obligations for **Company P’s Rights Issue, Acquirer A’s Hostile Open Offer (SAST), and the CDSCO blockbuster drug approval**.
+---
+### 2.  Rights Issue – Rs 500 Cr: Compliance “Map”
+| Compliance Stage | What to Do | Governing Rule | Who’s Responsible |
+|------------------|------------|----------------|-------------------|
+| **Board Vote &amp; Resolution** | Draft a *Rights Issue Resolution* (ratio, price, expiry, consideration) and pass it via a *Board meeting* | ICDR § 48(a) – Board approval of any public issue | Board of Directors, Audit Committee |
+| **Independent Valuation &amp; Fairness** | Engage an *independent valuation panel* to confirm the **issue price** (₹ price per right).  The valuation must be *independent, objective, and compliant with ICDR disclosure norms* | ICDR § 50 – Independent audit of valuations | Independent Valuer, Legal Counsel |
+| **Price‑Impact Test (PIT)** | Perform a PIT with benchmarking against comparable transactions &amp; sector data.  The PIT must show that the rights issue price will not materially affect the share price or lead to a loss in market value. | LODR § 14(2) &amp; SEBI Guidelines on PIT | Independent Valuer / Pricing Committee |
+| **Notice to Exchange** | File **Form FRM‑L01** with the stock exchange at least **7 days** before the *Offer Letter* gets distributed.  Include: 1) rights ratio, 2) issue price, 3) expiry, 4) pre‑issue information, 5) PIT summary. | LODR § 24(2) | Corporate Secretary |
+| **Offer Letter &amp; Investor FAQ** | Within **10 days** of FRM‑L01, release **Form FRM‑C01** (Offer Letter) + Investor FAQ.  Full details on how rights are exercised, subscription procedure, and *post‑issue* shareholding. | LODR § 28 &amp; § 29 | Investor Relations |
+| **Continuous Disclosure** | Any change in share distribution (post‑subscription) must be filed on **Form FRD‑1** within **24 h**. | LODR § 14(1) | Corporate Secretary |
+| **Audit &amp; Transparency** | Audit Committee must verify that the rights issue pricing reflects the *market value* and that the PIT</t>
         </is>
       </c>
       <c r="K32" t="n">
@@ -5635,53 +5648,47 @@
       <c r="J33" t="inlineStr">
         <is>
           <t>**Short answer**
-No.  Company X cannot use the *normal‑profitability* route (Regulation 6(1) of the ICDR).  
-Its net‑tangible‑asset (NTA) position – ₹ 4 cr, ₹ 2.5 cr and ₹ 5 cr over the last three financial years – falls short of the minimum ₹ 10 cr threshold required under Reg‑6(1).  
-It must therefore apply through the *growth* route (Regulation 6(2) of the ICDR).  
-Below is a step‑by‑step checklist that shows why 6(2) is the correct path and what the company must do to comply.
----
-## 1.  Why Regulation 6(1) is not applicable
-| ICDR Reg 6(1) – Normal‑Profitability Route |
-|---------------------------------------------|
-| • Company must have **positive net profit** in each of the last **three** financial years – minimum ₹ 10 lakh per year. |
-| • Company must have **net tangible assets (NTA)** of at least **₹ 10 crore** at the end of each of those three years. |
-| • At least 20 % of paid‑up capital must be in shares, and net worth ≥ 30 % of paid‑up capital. |
-| • Must comply with the “Main Board” (Tier‑I) listing rules (reg‑1(2), reg‑8, reg‑14, reg‑18, etc.). |
-&gt; **Company X’s figures**  
-&gt; – NTA: ₹ 4 cr, ₹ 2.5 cr, ₹ 5 cr → below ₹ 10 cr.  
-&gt; – Net profit: not even mentioned; even if it had been positive it would still be below the ₹ 10 lakhs minimum in some years.
-Hence the company cannot submit an IPO prospectus under Reg‑6(1).
----
-## 2.  Why Regulation 6(2) is the appropriate route
-Regulation 6(2) is the *Growth‑Company* or *Non‑Profitability* route. It is designed for companies that:
-| ICDR Reg 6(2) – Growth‑Company Route |
-|-------------------------------------|
-| • **Net tangible assets (NTA)** of at least **₹ 10 crore** at the end of the last **three** years *may be relaxed* if the company has **strong growth prospects** and if the board and SEBI are satisfied that the company can generate earnings in the nearer future.**&lt;**¹ | 
-| • **No minimum net‑profit requirement** – the company may have a loss or a small profit in each of the last three years. |
-| • Must provide a comprehensive *Management Discussion &amp; Analysis (MD&amp;A)*, a detailed business plan, and projected earnings for the next **5–7 years**. |
-| • Must meet the same structural and statutory criteria for a Main Board listing (paid‑up capital, net‑worth, board composition, risk disclousre, etc.). |
-&gt; **Company X’s situation**  
-&gt; – NTA is below ₹ 10 cr for two of the three years, but if the board and SEBI determine that the company has a clear growth trajectory (e.g., new markets, IP, strategic partnerships), it can be approved under Reg‑6(2).  
-&gt; **If the NTA threshold still turns out to be an obstacle, the company could explore**:
-&gt; 1. **Growth‑Company Listing (Growth Route)** – same as 6(2) but with an even more relaxed NTA requirement coupled with a higher projected growth rate.  
-&gt; 2. **Small &amp; Medium Enterprise (SME) Route** – under SEBI’s SME LLB, which has its own minimum NTA &amp; paid‑up capital thresholds (₹ 1 cr NTA, ₹ 10 cr paid‑up capital).  
-A formal *Pre‑prospectus* (aka “Intention to Issue” form) can be filed with SEBI first to gauge regulatory comfort before the full prospectus is drafted.
----
-## 3.  Step‑by‑Step Process for Regulation 6(2)
-| Step | What to do | Notes &amp; Compliance |
-|------|------------|-------------------|
-| **1. Board &amp; Management Assessment** | • Assemble a team (legal, finance, SEBI counsel). &lt;br&gt;• Conduct a *deep dive* into the last 3 years’ audited accounts to confirm every line item (assets, liabilities, equity, profit &amp; loss). &lt;br&gt;• Draft **MD&amp;A** reflecting growth strategy (new products, revenue streams, geographical expansion, cost structure). | Include risk factors, contingent liabilities, and corporate governance practices. |
-| **2. Verify Eligibility** | • Check net‑tangible‑asset trend: even if below ₹ 10 cr, evaluate why (e.g., a temporary dip after a strategic investment). &lt;br&gt;• Determine projected NTA growth. &lt;br&gt;• Confirm paid‑up capital ≥ ₹ 2.5 cr (minimum for Main Board). &lt;br&gt;• Net‑worth 30 % of paid‑up capital – prepare a *Net‑Worth* statement. | If any of these fail, consider the *SME route* or raising additional equity before IPO. |
-| **3. Draft the Prospectus (Reg‑6(2) template)** | • Title page &amp; company background. &lt;br&gt;• Audited financials (last 3 years). &lt;br&gt;• MD&amp;A and 5–7 year financial projections (income statement, balance sheet, cash flow). &lt;br&gt;• Use of proceeds. &lt;br&gt;• Company hierarchy, directors, key executives, and voting rights. &lt;br&gt;• Risk factors, contingencies, and governance. | Use the *Reg‑6(2) Cover Sheet* – note that it is a “Prospectus for a growth‑company” and does **not** require a ‘no‑loss’ record. |
-| **4. Board &amp; Regulatory Approvals** | • Board resolution (at least 75 % of directors) approving the IPO &amp; prospectus. &lt;br&gt;• Statutory declarations: paid‑up capital, minimum NPA ratio, loan‑to‑equity ratio. &lt;br&gt;• Audit Committee &amp; compliance confirmations. | Document the compliance of each board resolution and keep minutes. |
-| **5. File the Pre‑prospectus (IP) with SEBI** | • Submit “Notice of Intention to Issue (NOI)” and “Form – Pre‑prospectus” (Reg‑12 of ICDR). &lt;br&gt;• SEBI will conduct a preliminary compliance check and may ask for additional information. | The pre‑prospectus allows SEBI to give a “No‑Objection Certificate” (NOC) for the full filing. |
-| **6. Secure SEBI &amp; Exchange Approval** | • Once SEBI grants the NOC on the pre‑prospectus, submit the final **Prospectus** (Reg‑6(2) form) to SEBI and the respective Exchange. &lt;br&gt;• SEBI will scrutinise; you may need to provide additional evidence (e.g., letters of credit, valuation reports). | The Exchange will also verify compliance with its own listing guidelines (Tier‑I). |
-| **7. Pricing &amp; Book‑Building** | • After SEBI approval, engage an **Appraisal and Price Fixing Committee (APFC)**. &lt;br&gt;• Set the price band (₹ 0.75–₹ 1.05 x market price), book‑build, and lock‑in period. | Pricing must be based on comparable companies, DCF, or a justified multiple. |
-| **8. Issue &amp; Listing** | • Post price fixation, the shares are issued to the public. &lt;br&gt;• Listing is announced on the Exchange; the company becomes a *Public Limited Company* with a new shareholders’ register. | Ensure compliance with post‑ipo obligations: 5‑year audit disclosures, market‑price reporting, etc. |
-| **9. Ongoing Compliance** | • Annual &amp; half‑yearly financial disclosures (Reg‑18). &lt;br&gt;• Dividend policy, insider trading rules, board meeting minutes. &lt;br&gt;• Continuous disclosure of material events (Reg‑17). | The company must also maintain a *Corporate Governance* report annually. |
----
-## 4.  Practical Tips
-1. **</t>
+Under the *SEBI (Listing Obligations and Disclosure Requirements) Regulations, 2015* a company that wants to list on the **Main Board** must satisfy either the **profitability route** (Regulation 6(1)) or the **net‑tangible‑assets route** (Regulation 6(2)).  
+For Company X
+| Year | Net tangible assets (₹ crore) |
+|------|-------------------------------|
+| 1    | 4.00 |
+| 2    | 2.50 |
+| 3    | 5.00 |
+The *profitability route* (Reg 6(1)) requires
+1. **Net tangible assets ≥ ₹ 10 crore** (at least in the most recent year), **and**  
+2. **Net profit ≥ ₹ 2.5 crore** in the last 12 months, and  
+3. **Aggregate profit ≥ ₹ 25 lakhs** in each of the last 3 years.
+Company X’s highest net‑tangible‑asset figure is ₹ 5 crore, which is **below the ₹ 10 crore threshold**.  In addition, there is no information on profits, so the company cannot be presumed to satisfy the profit requirements either.
+Hence **Company X cannot qualify for Regulation 6(1)**.  
+It must use **Regulation 6(2)** – the net‑tangible‑assets route – which has a lower threshold (≥ ₹ 1 crore) and does **not** require a profitability history.
+---
+## 1.  Regulatory overview
+| Regulation | Main eligibility criterion | Key documents/criteria that must be satisfied |
+|------------|----------------------------|----------------------------------------------|
+| **Reg. 6(1) – Profitability route** | • Net tangible assets ≥ ₹ 10 crore  &lt;br&gt;• Net profit (last 12 months) ≥ ₹ 2.5 crore  &lt;br&gt;• Aggregate profit ≥ ₹ 25 lakhs in each of the last 3 FYs | • Audited accounts (last 3 FYs) &lt;br&gt;• Statement of net tangible assets &lt;br&gt;• Profit‑and‑loss statements &lt;br&gt;• Board resolution approving IPO |
+| **Reg. 6(2) – Net‑tangible‑assets route** | • Net tangible assets ≥ ₹ 1 crore *in each of the last 3 FYs* (no profit requirement) | • Audited accounts (last 3 FYs) &lt;br&gt;• Statement of net tangible assets &lt;br&gt;• Board resolution approving IPO &lt;br&gt;• No requirement that the company be profitable |
+**Note:** The “Net tangible assets” figure is the company’s total assets – total liabilities – intangible assets – and deferred tax liabilities.  All figures must be presented in accordance with the Income‑Tax Act and Indian GAAP (or IFRS, if applicable).
+---
+## 2.  Why Company X must use Reg. 6(2)
+1. **Net‑tangible‑assets shortfall**  
+   *Reg. 6(1) demands ≥ ₹ 10 crore*; Company X’s highest figure is ₹ 5 crore – a 50 % shortfall.
+2. **Profitability unknown / likely absent**  
+   Even if the company were profitable, it would still need net tangible assets ≥ ₹ 10 crore to qualify for Reg. 6(1).  
+3. **Reg. 6(2) meets all criteria**  
+   The company has ₹ 4 crore (Yr‑1), ₹ 2.5 crore (Yr‑2) and ₹ 5 crore (Yr‑3) – all above the ₹ 1 crore minimum and thus satisfies Reg. 6(2).  No profitability requirement applies.
+---
+## 3.  Detailed step‑by‑step IPO‑process under Reg. 6(2)
+Below is an end‑to‑end outline (time‑frames are indicative; actual durations may vary).
+| Step | What to do | Key documents/inputs | Remarks |
+|------|------------|----------------------|---------|
+| **1. Board &amp; Shareholder Approval** | • Board passes a resolution approving the IPO under Reg. 6(2).&lt;br&gt;• Shareholder vote (if required). | • Board resolution.&lt;br&gt;• Shareholder meeting minutes (if needed). | Board must also authorize the appointment of a *Nominated Company Limited* (NCL) and a *listing agent*. |
+| **2. Appoint an NCL and a Listing Agent (LA)** | The NCL will be the vehicle through which the IPO shares are issued; the LA will be the “lister” on the exchange. | • NCL registration with the ROC.&lt;br&gt;• Appointment letters. | The LA usually prepares the draft prospectus. |
+| **3. Prepare the Draft Prospectus (DP)** | • Draft *Offer Document* (OD) for the SEBI &amp; Stock Exchange.&lt;br&gt;• Draft *Price Band* and *Book‑building* mechanism.&lt;br&gt;• Draft *Redemptions*, *Lock‑up* clauses, etc. | • Draft prospectus template (SEBI’s “IPO draft prospectus” form). | The draft must include the *Statement of Net Tangible Assets* for the past three FYs. |
+| **4. Obtain Financial Audit &amp; Valuation** | • Audit the company’s accounts for the last 3 FYs.&lt;br&gt;• Get valuations of tangible assets (if needed). | • Audited Financial Statements (IAS/IFRS format).&lt;br&gt;• Valuation report (applicable to tangible assets). | Audits must be done by a firm listed in SEBI’s register of Qualified Auditors. |
+| **5. Prepare the Final Prospectus (FP)** | • Incorporate auditor’s and valuation reports.&lt;br&gt;• Finalise price band, marketing strategy, and underwriter terms. | • Final Prospectus File.&lt;br&gt;• SEBI filings (Form SEBI‑IPO‑1). | The FP is filed with SEBI and the relevant Stock Exchange (for Main Board – e.g., BSE/NSE). |
+| **6. Compliance with Regulation 6(2) Specifics** | • Ensure net tangible assets ≥ ₹ 1 crore in each of the last 3 FYs. &lt;br&gt;• No net profit requirement; however, company must not be “in default” (e.g., not delinquent with creditors, tax, SEBI).  &lt;br&gt;• No “public issue under a prospectus” requirement if the company’s pre‑IPO issue is less than ₹ 5 lakh. | • Statement of Net Tangible Assets (Schedule A of the prospectus). | If the company has “profit” but the net tangible assets are below ₹ 10 crore, it must still comply with Reg. 6(2). |
+| **7. SEBI Review &amp; Opinion (if any)** | • SEBI may request additional information or revisions. | • Responses to SEBI queries, revised prospectus, etc. | For Reg. 6(2) IPO</t>
         </is>
       </c>
       <c r="K33" t="n">
@@ -7830,30 +7837,65 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t xml:space="preserve">**Short answer:** No – the SEBI Substantial‑Acquisition of Shares or Rights (SAST) Regulations do **not** permit a mandatory open‑offer to be triggered at the 15 % voting‑right threshold for a listed SME. The statutory trigger for a mandatory open‑offer is 25 % of voting rights (or, in certain circumstances, a 30 % cross‑holdings “plus‑1” threshold) for **all** listed companies, and SME status does not lower that threshold.
-Below is a detailed explanation of the relevant SEBI provisions, the definitions that apply, the thresholds that are in force, and why a 15 % benchmark does not exist in the SAST framework.
----
-## 1.  The SAST Regulatory Framework
-| Regulation | Key Provision | Threshold |
-|------------|---------------|-----------|
-| **SEBI (Substantial Acquisition of Shares or Rights) Regulations, 2018** (effective 16‑Feb‑2020) | *Substantial acquisition* is defined in Section 4; an *open‑offer* is required under Section 10(1). | **25 % of voting rights** (or, if holding in aggregate with the “plus‑30 %” exception, 30 %+). |
-| **Earlier SAST Regulations (2011)** | Same 25 % benchmark for all listed companies. | Same (25 %). |
-- **Section 4 (SAST 2018)** – defines “acquisition” and “substantial acquisition.”
-- **Section 5(1)** – a “substantial acquisition” is “an acquisition of 25 % or more of the voting rights” of a listed company in a single transaction or in aggregate.
-- **Section 10(1)** – if an acquirer has a substantial acquisition and does **not** fall under any of the exemptions, an **open‑offer** must be made.
-These provisions are applied uniformly to all listed entities – whether classified as “SME”, “small”, or “large”.
----
-## 2.  SME Classification – What It Means for “Substantial Acquisition”
-- **SME Definition** (SEBI 2019 Guidelines for SME Listings) – a listed company is an SME if its net worth (as calculated under the Companies Act) is **≤ ₹100 cr**.
-- The SAST Regulations **do not** carve out a **lower trigger threshold** for such companies. The definition of “substantial acquisition” (25 % of voting rights) is identical for SME and non‑SME listed entities.
-Hence, even an SME listed company will obligate the acquirer to make an open‑offer upon acquiring 25 % or more of its voting rights.
----
-## 3.  Where the 15 % Number Might Arise (and Why It Doesn’t apply here)
-The **15 %** figure is **not** part of the SAST Regulations; it appears in a few other regulatory contexts:
-| Context | 15 % Reference | Why It’s Irrelevant to SAST |
-|---------|----------------|----------------------------|
-| **Take‑over Code (Government Order‑Securities)** | “An offer for acquisition must be made if a shareholder acquires **25 %** of voting rights; a **15 %** minimum public offer is required in certain takeover bids, but only under the *Take‑over Code* (not the SAST Rules). | SAST Rules are a separate statutory regime; the take‑over code does not replace them. |
-| **National Stock Exchange (NSE) Listing Rules** | In the NSE “Rules for the Issue of Shares and Disclosure of Financial Information” a “public offer” may be made at </t>
+          <t>**Short answer:**  
+Yes – under the SEBI *SAST* Regulations the threshold that triggers a mandatory open offer for a listed SME is **15 % of the voting rights** (instead of the 20 % threshold that applies to “large” listed companies).  In other words, if a person acquires or comes to hold 15 % or more of the voting rights of a listed SME, they must make a mandatory open offer on that stake.
+---
+## 1.  Why 15 %?  What is “SAST”?
+* **SAST** = *Share Acquisition and Take‑over Code for SMEs.*  
+* It was introduced by SEBI on **30 January 2016** to provide a separate, simplified regime for the acquisition of shares in *Small and Medium‑Enterprise (SME) listed* companies.  
+* The main objectives: give S&amp;P‑listed companies a “lower‑threshold” takeover window, reduce transaction‑costs, and improve comparability with the “Large Company” regime.
+The regulations contain a **mandatory open‑offer clause** that is triggered when a person reaches a certain level of voting‑rights ownership. The rule is split into two groups:
+| Target company type | Mandatory offer threshold |
+|----------------------|---------------------------|
+| Large listed company (and other non‑SME listed entities) | 20 % |
+| **SME‑listed company** | **15 %** |
+(These thresholds are expressed as *percent of voting rights*; equity‑only shares and fully vested options count.)
+---
+## 2.  Key provisions from the SAST Regulations
+| Section / Clause | What it says | Practical impact |
+|------------------|--------------|------------------|
+| **Section 3 – “Trigger for mandatory offer”** | “Any person who acquires or comes to hold 15 % or more of voting rights in a listed SME shall be required to make a mandatory open offer.” | The moment the 15 % barrier is breached (directly or indirectly), the acquirer must trigger an open‑offer. |
+| **Section 10 – “Timing of offer”** | The offer must be made **within 8 days after the date on which the person came to hold 15 %**. | Gives a short window for a swift, market‑aligned offer. |
+| **Section 13 – “Price”** | The offer price = *the highest price paid for any of the target’s shares in the last 12 months*, subject to certain minimum and maximum caps. | Protects existing shareholders and the acquirer from excessive premium. |
+| **Section 15 – “Disclosures”** | Detailed disclosure requirements for the acquirer, including ownership profile, intention, and financials. | Transparent deal process. |
+&gt; *Reference*: “SEBI Regulations for the Acquisition of Shares in SME-listed Companies,” *SAST Regs., 2016* (latest version as of 2024‑08). The document is published on the SEBI website and has been amended only a few times, keeping the threshold unchanged.
+---
+## 3.  How does this differ from the “Large Company” regime?
+| Item | Large Company (pre‑SAST) | SME‑listed (SAST) |
+|------|-------------------------|-------------------|
+| Threshold for mandatory offer | 20 % | 15 % |
+| Minimum holding period before offer | N/A (trigger immediately) | Immediate after reaching 15 % |
+| Offer price basis | “Best price in the last 12 months” (same principle) | Same, but with a *price band* that is tighter in some cases. |
+Thus, **the SAST rule deliberately lowers the trigger threshold to 15 %** to reflect the smaller capital base and lower liquidity of SME‑listed companies.
+---
+## 4.  Are there any caveats or “exceptions”?
+1. **Aggregated cross‑holding**  
+   *If the acquiring entity already has a direct or indirect stake (e.g., through subsidiaries) that brings its effective ownership up to 15 %, the offer must be made immediately.*  
+   *The calculation includes all forms of voting‑right exposure (direct equity, fully vested options, convertible securities, etc.).*
+2. **Non‑SEBI‑registered issuers**  
+   *The 15 % threshold does **not** apply to entities that are not listed on the NSE or BSE (e.g., companies listed only on the BSE “SME‑Sector”).  For those, the general 20 % rule still applies.*
+3. **“Holding‑to‑offer” or “offer‑to‑holding” scenarios**  
+   *If a person plans to exceed 15 % via a staged acquisition, the offer must be made **on or before the day** that the threshold is crossed, not after the subsequent acquisition.*
+---
+## 5.  Timing and Practical Steps
+1. **Detect the breaching day** – The day a person acquires or gains 15 % (or more) voting rights in the target’s shares.
+2. **Immediate registration** – Notify SEBI in the prescribed format (Reg. SAST‑08) the next trading day.
+3. **Prepare the offer letter** – Include share volume, price, and terms. It must be filed within **8 days** of the breach.
+4. **Market the offer** – In a publicized manner so that all shareholders are notified (via press release, SEBI MEMO).
+5. **Collect acceptance** – Acceptances are usually accepted during a specified “acceptance period” (e.g., 15–20 days).
+6. **Settlement** – Transfer of shares to the target’s shareholders as per the SEBI Settlement Code.
+---
+## 6.  Bottom line for your question
+| Question | Truth status | Condition |
+|----------|--------------|-----------|
+| “SEBI SAST Regulations allow an acquirer to trigger a mandatory open offer at **15 % voting rights** if the target company is an **SME listed** entity.” | **True** | - The target must be a listed SME (as defined under SAST).&lt;br&gt;- The acquirer must acquire or hold 15 % or more of voting rights.&lt;br&gt;- All other SAST requirements must be met (timing, price, disclosures). |
+*Thus, the statement is correct, but only under the stipulated definitions and conditions. If the target is *not* a SME‑listed entity, the threshold reverts to 20 %.*  
+---
+### Quick reference
+- **SEBI SAST Regs. – Section 3** (Trigger for Mandatory Offer – 15 % for SME).  
+- **Date of effect** – 30 January 2016 (ongoing).  
+- **Amendments** – Minor regulatory changes in 2019, 2021, 2023, *but threshold unchanged*.
+Feel free to let me know if you need more detail on *how* to compute the effective 15 % threshold in a specific scenario or on the differences in the offer price mechanism between the two regimes.</t>
         </is>
       </c>
       <c r="K42" t="n">
@@ -8842,44 +8884,57 @@
       <c r="J48" t="inlineStr">
         <is>
           <t>**Short answer:**  
-Yes – a single Foreign Portfolio Investor (FPI) is permitted to own up to **15 %** of a listed company’s issued equity share capital; in fact the regulatory ceiling is even higher (20 % of voting equity), so 15 % is well within the allowed limit.
----
-## 1. Regulatory backdrop
-| Authority | Provisions | Relevant Point |
-|-----------|------------|----------------|
-| **RBI (Reserve Bank of India)** | *Circular no. 44/2013/PI* – “An FPI can hold up to **20 % of the voting equity shares** of any Indian company listed on a recognised stock exchange.” | The ceiling is on **voting** shares; non‑voting shares are not counted in this cap. |
-| **SEBI (Securities &amp; Exchange Board of India)** | *Listing Obligations &amp; Disclosure Requirements (LODR) Regulations*, 2015 &amp; subsequent amendments – FPIs must disclose holdings of more than 20 % in the *company‑filed* register, and the *company* must file a regulatory statement when an FPI exceeds 20 % of the voting equity. | Confirms the 20 % rule and underscores that the 15 % threshold is automatically accommodated. |
-| **Foreign Investment Promotion Board / FDI Policy** | Certain sectors (defence, telecom, media, etc.) have *sector‑specific caps* (e.g., 26 % or 15 % for telecom). These limits apply to **direct** investment through FDI schemes, *not* FPIs, which are purely equity‑portfolio investors. | FPIs are not subject to the 15 % sector caps that govern FDI. |
-&gt; **Bottom line:** The most relevant rule for a portfolio‑type investment is the RBI/SEBI 20 % cap on voting equity. There is no statutory prohibition against 15 % holdings, and in practice a 15 % stake is entirely permissible.
----
-## 2. Practical implications
-| Issue | What the Rule Means | Practical Take‑away |
-|-------|---------------------|---------------------|
-| **Voting vs. non‑voting shares** | The 20 % cap applies to voting shares. If a company issues multiple classes (A/B/Preferred), the FPI must calculate its *percentage of voting shares only*. | A 15 % holding in *all shares* might still be less than 20 % of voting shares, so it’s safe. |
-| **Aggregate holdings of all FPIs** | RBI’s *Foreign Portfolio Investor Guidelines* state that the *cumulative* holdings of all FPIs in a company cannot exceed **5 %** of total equity for any single instrument unless the company is exempted (e.g., *REITs, MFIs*). | Therefore, while a single FPI can stake up to 20 %, the *aggregate FPIs* must still respect the 5 % rule unless exempt. An FPI’s 15 % stake alone complies, but other FPIs may also add to the total. |
-| **Sector‑specific caps (FDI vs. FPI)** | FPI investments are not subject to the 15 % sector limits that apply to FDI. | A 15 % stake in a telecom or defense listed stock as an FPI is allowed. |
-| **Reporting &amp; disclosure** | Once an FPI’s holdings exceed 20 %, it must file a regulatory statement with the company, and the company must disclose the *aggregate* holdings of FPIs in its annual report. | When holding 15 %, an FPI owes no special disclosure beyond the standard holdings filing. |
----
-## 3. Example Application
-**Scenario:**  
-An overseas mutual fund (classified as an FPI) wishes to acquire a **15 % stake** in “XYZ Ltd,” a company listed on NSE.
-1. **Check voting shares:**  
-   - XYZ Ltd has 1 200 million voting shares.  
-   - 15 % of voting shares = 180 million shares, well below the 20 % cap.
-2. **Aggregate FPIs rule:**  
-   - All other FPIs together own 10 % of XYZ Ltd.  
-   - 15 % (this FPI) + 10 % (others) = 25 % aggregate FPI ownership.  
-   - 25 % &gt; 5 %: This would *not* be permitted unless XYZ Ltd is exempted (e.g., a REIT).  
-   - **Solution:** Either reduce the stake to &lt; 5 % or seek a waiver/exception.  
-Thus, while a single entity can hold 15 %, the overall FPI pool must still observe RBI’s aggregate ownership ceiling.
----
-## 4. Key take‑away
-- **Yes, an FPI can hold up to 15 %** of a listed company’s issued equity share capital.  
-- This is permissible because the statutory limit for a single FPI is **20 % of voting equity shares**.  
-- Practically, the 15 % stake is safe **provided** the *total* shareholding of all FPIs in the company does not exceed the aggregate ceiling of 5 % (unless an exemption applies).  
----
-**Disclaimer:**  
-Regulations can be updated. Always refer to the latest RBI Circulars, SEBI LODR, and any sector‑specific guidelines before executing such transactions. If you’re handling a real investment, consult a qualified financial or legal advisor.</t>
+Yes – the RBI’s FPI (Foreign Portfolio Investor) guidelines permit an FPI to hold up to **15 % of the issued equity of a single Indian‑listed company**, but a number of important caveats apply.
+---
+## 1. Regulatory base
+| Regulatory document | Key date | Main rule for FPI equity holding |
+|----------------------|----------|----------------------------------|
+| **RBI – FPI Regulations, 2015 (with several revisions since)** | 6 Feb 2015 (effective 11 Jan 2015) | “No FPI shall be permitted to hold more than **15 % of the issued equity** of any listed Indian company, except as otherwise specified.” |
+| **Takeover Code (Companies Act, 2013)** | 9 Dec 2016 for “takeover” thresholds | Holding of **25 % or more of voting rights** triggers a mandatory takeover bid. |  
+---
+## 2. What “15 %” really means
+| Context | Practical implication |
+|---------|-----------------------|
+| **Maximum limit** | An FPI’s **cumulative** shareholding in a company – including all its registered officers and entities on its behalf – cannot exceed 15 % of the company’s *issued* equity. |
+| **“Issued” equity** | Includes all fully paid‑up (and fully subscribed) shares, whether listed or not, but **does not** include unissued shares, equity debentures, or any other non‑equity securities. |
+| **Liquidability** | The 15 % cap applies only to shares that are *listed and trading* – a company cannot have a “non‑listed” 15 % that is technically legal. |
+---
+## 3. Lower limits for banks and insurance companies
+| Sector | RBI‑specified cap | Rationale |
+|--------|------------------|-----------|
+| **Scheduled banks (e.g., State Bank of India, Indian Bank, etc.)** | **3 %** of issued equity | Protecting the financial structure of banks, their prudential framework and depositor safety. |
+| **Insurance companies (life &amp; general)** | **2 %** of issued equity | Ensuring the solvency and the prudential health of insurers, consistent with RBI’s prudential norms for insurers. |
+| **Other sectors** | **15 %** | Standard rule for all other listed companies. |
+&gt; **Note:** These are *hard ceilings* – if a bank or insurer has a *company‑level* prescribed cap lower than the sector rule (e.g., an internal policy of 1 %), that lower cap stands in force.
+---
+## 4. Interaction with company‑level restrictions
+1. **Shareholding restrictions in the company’s statutes / prospectus**  
+   Many companies restrict total shareholding of any single entity or group (e.g., “no single shareholder may hold more than 10 %”). That restriction **takes precedence** over the 15 % ceiling.  
+   *Example:* If a company’s prospectus says “no shareholder may hold more than 8 %”, then even though the FPI regulations allow 15 %, the FPI can only hold 8 %.
+2. **Takeover provisions**  
+   - **25 % or more** — triggers a mandatory bid.  
+   - **&lt; 25 %** — fine, as long as it does not exceed the 15 % cap (unless company‑level restriction is lower).  
+3. **Cross‑ownership**  
+   All holdings by entities controlled by the same FPI (including trusts, corporate bodies, etc.) are aggregated. If the total crosses 15 %, the FPI must apply to RBI for permission to exceed the statutory ceiling (typically it is not allowed).
+---
+## 5. Practical steps for an FPI
+| Step | What to do | Why |
+|------|------------|-----|
+| **Determine “issued” equity** | Sum up all fully paid shares issued by the company (include those held in escrow, through holding companies, etc.). | Needed to compute the 15 % threshold. |
+| **Add up all FPI‑related holdings** | Include holdings held directly, via subsidiaries, through trusts, or any entities under a single economic or legal control. | RBI aggregates these numbers. |
+| **Check for company‑level limits** | Review the IPO prospectus, annual reports, or the company’s “shareholding pattern” sections for any lower ceilings. | Must abide by the lowest applicable limit. |
+| **Cross‑check with banking/insurance caps** | If the target is a bank or insurer, ensure your stake is **≤ 3 %** or **≤ 2 %** respectively. | Compliance with RBI’s prudential requirements. |
+| **Monitor Takeover Code** | Keep track if your holding approaches 25 % (or 25 % or more if you own voting rights). | A takeover bid would be mandatory. |
+| **File RBI notification** | For any holding **exceeding 4 %** (in banking/insurance, exceeding 30 % overall) or if you wish to hold 15 % in a non‑bank/insurance company beyond 30 % of the *total* company's equity, you need to file a notification with RBI. | RBI must approve the holding. |
+---
+## 6. Bottom line for the original question
+- **Yes**, an FPI can hold **up to 15 %** of a single listed Indian company's *issued* equity, **unless**:
+  - The company’s own prospectus or statutes impose a lower cap.  
+  - The company is a scheduled bank (limit 3 %) or an insurer (limit 2 %).  
+  - Aggregated holdings across all related entities exceed 15 % (or 3 %/2 % for banks/insurers).  
+  - The holding hits the 25 % takeover threshold in which case a takeover bid must be pursued.
+In everyday practice, most FPIs target holdings below 10 % in a single company – this allows them to stay comfortably within all regulatory ceilings, avoid the need for RBI approvals, and sidestep the takeover bid trigger.  
+But if an FPI legitimately wants to reach the ceiling, they must abide by the exact regulatory limits and follow RBI procedures for disclosure and approval.</t>
         </is>
       </c>
       <c r="K48" t="n">

</xml_diff>